<commit_message>
Merged PR 2272: Merge applicationintake-refactoring to master
Updated changes till date
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AA5F0FA-57CB-4FB0-8C90-E966F47EC32F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10CDBDFE-6E5E-4C07-90AE-6D2F8376CD51}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="40">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -116,15 +116,6 @@
     <t>Primary</t>
   </si>
   <si>
-    <t>deep@vana.com</t>
-  </si>
-  <si>
-    <t>Jim</t>
-  </si>
-  <si>
-    <t>Cobat</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Automation Organization Test</t>
   </si>
   <si>
@@ -138,6 +129,27 @@
   </si>
   <si>
     <t>USA</t>
+  </si>
+  <si>
+    <t>automation.jim@yopmail.com</t>
+  </si>
+  <si>
+    <t>Address1__c</t>
+  </si>
+  <si>
+    <t>MailingCity</t>
+  </si>
+  <si>
+    <t>MailingState</t>
+  </si>
+  <si>
+    <t>MailingPostalCode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation </t>
+  </si>
+  <si>
+    <t>Contact</t>
   </si>
 </sst>
 </file>
@@ -162,20 +174,32 @@
     </font>
     <font>
       <sz val="7"/>
-      <color rgb="FF222222"/>
-      <name val="Consolas"/>
-      <family val="3"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE3F3FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -183,12 +207,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE0E3E5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE0E3E5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE0E3E5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE0E3E5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -197,7 +236,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -540,7 +584,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -551,7 +595,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -562,7 +606,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -775,7 +819,7 @@
         <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -786,7 +830,7 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -811,7 +855,7 @@
         <v>9908786788</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -819,10 +863,10 @@
         <v>26</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -830,51 +874,51 @@
         <v>34</v>
       </c>
       <c r="C7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
-      </c>
       <c r="C8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" t="s">
-        <v>14</v>
+      <c r="B9" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="B10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10">
+        <v>20171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11">
-        <v>20171</v>
+      <c r="B11" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merged PR 2305: Merge applicationintake-refactoring to master
today fixes.
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9935532-93D1-4498-9512-962FD758F76D}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12F98B9B-9296-4121-B36B-E98BD53E1E48}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="5" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="1" r:id="rId1"/>
@@ -143,13 +143,13 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>IADO</t>
-  </si>
-  <si>
-    <t>InAuOrg1</t>
-  </si>
-  <si>
-    <t>Product Automation Org</t>
+    <t>Product Automation permanent</t>
+  </si>
+  <si>
+    <t>PROrg1</t>
+  </si>
+  <si>
+    <t>IADPO</t>
   </si>
 </sst>
 </file>
@@ -584,7 +584,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -606,7 +606,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -617,7 +617,7 @@
         <v>7</v>
       </c>
       <c r="C5">
-        <v>915927646</v>
+        <v>925927646</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Merged PR 2335: Merge planningmodulenewscenarios to master
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12F98B9B-9296-4121-B36B-E98BD53E1E48}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF70F737-C1C7-453A-8078-6F4D9ACA0B0F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="5" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="1" r:id="rId1"/>
@@ -143,13 +143,13 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>Product Automation permanent</t>
-  </si>
-  <si>
-    <t>PROrg1</t>
-  </si>
-  <si>
-    <t>IADPO</t>
+    <t>Product Automation permanent Orgtn</t>
+  </si>
+  <si>
+    <t>PROrgtn1</t>
+  </si>
+  <si>
+    <t>IADOPO</t>
   </si>
 </sst>
 </file>
@@ -617,7 +617,7 @@
         <v>7</v>
       </c>
       <c r="C5">
-        <v>925927646</v>
+        <v>926927646</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -633,7 +633,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fixed Home Test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -1,24 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF70F737-C1C7-453A-8078-6F4D9ACA0B0F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BEBDA5B-ACD4-46F4-8775-E8EB58592FB2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="4" activeTab="7" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="1" r:id="rId1"/>
-    <sheet name="Edition" sheetId="2" r:id="rId2"/>
-    <sheet name="AdditioanlAddressesCreation" sheetId="3" r:id="rId3"/>
-    <sheet name="AdditioanlAddressesEdition" sheetId="4" r:id="rId4"/>
-    <sheet name="RelatedContactsCreation" sheetId="5" r:id="rId5"/>
-    <sheet name="RelatedContactsEdition" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="7" r:id="rId2"/>
+    <sheet name="Edition" sheetId="2" r:id="rId3"/>
+    <sheet name="AdditioanlAddressesCreation" sheetId="3" r:id="rId4"/>
+    <sheet name="AdditioanlAddressesEdition" sheetId="4" r:id="rId5"/>
+    <sheet name="RelatedContactsCreation" sheetId="5" r:id="rId6"/>
+    <sheet name="RelatedContactsEdition" sheetId="6" r:id="rId7"/>
+    <sheet name="New IDC" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="48">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -150,6 +152,30 @@
   </si>
   <si>
     <t>IADOPO</t>
+  </si>
+  <si>
+    <t>CostRate__c</t>
+  </si>
+  <si>
+    <t>Budget_Categories__c</t>
+  </si>
+  <si>
+    <t>PeriodFrom__c</t>
+  </si>
+  <si>
+    <t>PeriodTo__c</t>
+  </si>
+  <si>
+    <t>IndirectCostRateType__c</t>
+  </si>
+  <si>
+    <t>New IDC</t>
+  </si>
+  <si>
+    <t>Personell</t>
+  </si>
+  <si>
+    <t>Final</t>
   </si>
 </sst>
 </file>
@@ -227,7 +253,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -242,6 +268,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -638,6 +665,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88396F45-2FFF-4754-A21D-9B04C546541E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06A9DB05-0B00-4A98-9FC7-C651680BE6AA}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -674,7 +710,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49FFA402-44F3-4194-95BC-AF87BBB9EC62}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -754,7 +790,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E2F0B9B-0D1C-441E-8138-8347B90B311F}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -791,7 +827,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ED4E39D-6BA6-4D31-BCA1-B2F0B4803773}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -930,7 +966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EEEF9E7-7E28-440F-BBD4-8BA71C7E537F}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -964,4 +1000,96 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAC09EB0-D87C-4E41-BE46-78AEA78D54B3}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="6">
+        <v>43738</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="6">
+        <v>43799</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Merged PR 2883: Merge Deepika_prod to master
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -1,24 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF70F737-C1C7-453A-8078-6F4D9ACA0B0F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BEBDA5B-ACD4-46F4-8775-E8EB58592FB2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="4" activeTab="7" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="1" r:id="rId1"/>
-    <sheet name="Edition" sheetId="2" r:id="rId2"/>
-    <sheet name="AdditioanlAddressesCreation" sheetId="3" r:id="rId3"/>
-    <sheet name="AdditioanlAddressesEdition" sheetId="4" r:id="rId4"/>
-    <sheet name="RelatedContactsCreation" sheetId="5" r:id="rId5"/>
-    <sheet name="RelatedContactsEdition" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="7" r:id="rId2"/>
+    <sheet name="Edition" sheetId="2" r:id="rId3"/>
+    <sheet name="AdditioanlAddressesCreation" sheetId="3" r:id="rId4"/>
+    <sheet name="AdditioanlAddressesEdition" sheetId="4" r:id="rId5"/>
+    <sheet name="RelatedContactsCreation" sheetId="5" r:id="rId6"/>
+    <sheet name="RelatedContactsEdition" sheetId="6" r:id="rId7"/>
+    <sheet name="New IDC" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="48">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -150,6 +152,30 @@
   </si>
   <si>
     <t>IADOPO</t>
+  </si>
+  <si>
+    <t>CostRate__c</t>
+  </si>
+  <si>
+    <t>Budget_Categories__c</t>
+  </si>
+  <si>
+    <t>PeriodFrom__c</t>
+  </si>
+  <si>
+    <t>PeriodTo__c</t>
+  </si>
+  <si>
+    <t>IndirectCostRateType__c</t>
+  </si>
+  <si>
+    <t>New IDC</t>
+  </si>
+  <si>
+    <t>Personell</t>
+  </si>
+  <si>
+    <t>Final</t>
   </si>
 </sst>
 </file>
@@ -227,7 +253,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -242,6 +268,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -638,6 +665,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88396F45-2FFF-4754-A21D-9B04C546541E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06A9DB05-0B00-4A98-9FC7-C651680BE6AA}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -674,7 +710,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49FFA402-44F3-4194-95BC-AF87BBB9EC62}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -754,7 +790,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E2F0B9B-0D1C-441E-8138-8347B90B311F}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -791,7 +827,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ED4E39D-6BA6-4D31-BCA1-B2F0B4803773}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -930,7 +966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EEEF9E7-7E28-440F-BBD4-8BA71C7E537F}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -964,4 +1000,96 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAC09EB0-D87C-4E41-BE46-78AEA78D54B3}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="6">
+        <v>43738</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="6">
+        <v>43799</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Merged PR 2989: Merge Deepika09may to master
Fixed test cases in Home
Created and Automated 6 new testcases in Negotiations
34331
58034
58032
58031
58030
58029
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B109CDA1-672E-49A1-90D4-4D046BED7F49}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4266E163-043A-45D6-820A-3432CAC1A61C}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="3" activeTab="3" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="3" activeTab="5" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="1" r:id="rId1"/>
@@ -208,7 +208,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -217,38 +217,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFE3F3FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFE0E3E5"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFE0E3E5"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFE0E3E5"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFE0E3E5"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -267,7 +246,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -276,14 +255,8 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -817,7 +790,7 @@
       <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="5" t="s">
         <v>48</v>
       </c>
       <c r="C8" t="s">
@@ -931,7 +904,7 @@
         <v>9908786788</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -942,55 +915,55 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" t="s">
         <v>31</v>
       </c>
       <c r="C7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" t="s">
         <v>32</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" t="s">
         <v>33</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" t="s">
         <v>34</v>
       </c>
       <c r="C10">
         <v>20171</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" t="s">
         <v>28</v>
       </c>
       <c r="C11" t="s">
@@ -1103,7 +1076,7 @@
       <c r="B5" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="4">
         <v>43738</v>
       </c>
     </row>
@@ -1114,7 +1087,7 @@
       <c r="B6" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="4">
         <v>43799</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed home test cases and removed refresh the page step from fetaure files
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4266E163-043A-45D6-820A-3432CAC1A61C}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFF70623-A80B-4425-BC41-C60B77E23EFB}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="3" activeTab="5" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="4" activeTab="7" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="1" r:id="rId1"/>
@@ -185,7 +185,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,28 +201,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="7"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE3F3FF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -230,23 +218,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FFE0E3E5"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFEDEDED"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -256,9 +233,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -706,7 +680,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -722,7 +696,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
@@ -733,7 +707,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -744,7 +718,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -755,7 +729,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
         <v>15</v>
@@ -766,7 +740,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
@@ -775,9 +749,9 @@
         <v>20171</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B7" t="s">
         <v>17</v>
@@ -786,11 +760,11 @@
         <v>29467</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
         <v>48</v>
       </c>
       <c r="C8" t="s">
@@ -826,7 +800,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
@@ -862,7 +836,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>22</v>
@@ -873,7 +847,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
         <v>23</v>
@@ -884,7 +858,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
@@ -895,7 +869,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
         <v>25</v>
@@ -906,7 +880,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
         <v>26</v>
@@ -917,7 +891,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B7" t="s">
         <v>31</v>
@@ -928,7 +902,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B8" t="s">
         <v>32</v>
@@ -939,7 +913,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B9" t="s">
         <v>33</v>
@@ -950,7 +924,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B10" t="s">
         <v>34</v>
@@ -961,7 +935,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B11" t="s">
         <v>28</v>
@@ -1001,7 +975,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>25</v>
@@ -1038,7 +1012,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -1049,7 +1023,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
         <v>40</v>
@@ -1060,7 +1034,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>41</v>
@@ -1071,7 +1045,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
         <v>42</v>
@@ -1082,7 +1056,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
         <v>43</v>
@@ -1093,7 +1067,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B7" t="s">
         <v>44</v>

</xml_diff>

<commit_message>
refactored home and org site visits and desk review
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22325"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B810DAE2-C698-4ECD-A4EC-A42E4B0D5687}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06BC9F1-099A-41EA-A78F-0BFB412B6992}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="4" activeTab="7" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="1" r:id="rId1"/>
@@ -139,9 +139,6 @@
     <t>MailingPostalCode</t>
   </si>
   <si>
-    <t xml:space="preserve">Automation </t>
-  </si>
-  <si>
     <t>Contact</t>
   </si>
   <si>
@@ -169,13 +166,16 @@
     <t>IndirectCostRateType__c</t>
   </si>
   <si>
+    <t>Final</t>
+  </si>
+  <si>
+    <t>Personnel</t>
+  </si>
+  <si>
+    <t>Automation Runtime</t>
+  </si>
+  <si>
     <t>New IDC</t>
-  </si>
-  <si>
-    <t>Final</t>
-  </si>
-  <si>
-    <t>Personnel</t>
   </si>
 </sst>
 </file>
@@ -578,7 +578,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -589,7 +589,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -600,7 +600,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -834,7 +834,7 @@
         <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -845,7 +845,7 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1010,7 +1010,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1018,7 +1018,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3">
         <v>20</v>
@@ -1029,10 +1029,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1040,7 +1040,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -1051,7 +1051,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -1062,10 +1062,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
         <v>44</v>
-      </c>
-      <c r="C7" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modification as per grantor regression
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A8A87A-CBAE-453A-90F6-A3F5A8CDB6FA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{938EDAA3-1C44-4F16-840B-883887063E34}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4097" yWindow="1029" windowWidth="16457" windowHeight="8554" firstSheet="4" activeTab="5" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="4" activeTab="7" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="49">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -176,13 +176,16 @@
   </si>
   <si>
     <t>Automation Runtime Contact</t>
+  </si>
+  <si>
+    <t>fieldName</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -200,6 +203,12 @@
     </font>
     <font>
       <sz val="7"/>
+      <color rgb="FF222222"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="5"/>
       <color rgb="FF222222"/>
       <name val="Consolas"/>
       <family val="3"/>
@@ -226,7 +235,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -236,6 +245,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -552,14 +562,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED470BA6-8708-4CF0-B2C5-EF741B2578C9}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.23046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -570,7 +580,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -581,7 +591,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -592,7 +602,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -603,7 +613,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -614,7 +624,7 @@
         <v>926927646</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -634,7 +644,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88396F45-2FFF-4754-A21D-9B04C546541E}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -643,14 +653,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06A9DB05-0B00-4A98-9FC7-C651680BE6AA}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="8.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -661,7 +671,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -680,13 +690,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49FFA402-44F3-4194-95BC-AF87BBB9EC62}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="14.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -697,7 +707,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -708,7 +718,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -719,7 +729,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -730,7 +740,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -741,7 +751,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -752,7 +762,7 @@
         <v>20171</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -760,7 +770,7 @@
         <v>17</v>
       </c>
       <c r="C7">
-        <v>29467</v>
+        <v>2946</v>
       </c>
     </row>
   </sheetData>
@@ -772,14 +782,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E2F0B9B-0D1C-441E-8138-8347B90B311F}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="8.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.53515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -790,7 +800,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -809,13 +819,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ED4E39D-6BA6-4D31-BCA1-B2F0B4803773}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="13.3046875" customWidth="1"/>
-    <col min="3" max="3" width="26.23046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
+    <col min="3" max="3" width="26.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -826,7 +836,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -837,7 +847,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -848,7 +858,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -859,7 +869,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -870,7 +880,7 @@
         <v>9908786788</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -881,7 +891,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -892,7 +902,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -903,7 +913,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -914,7 +924,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -925,7 +935,7 @@
         <v>20171</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -948,13 +958,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EEEF9E7-7E28-440F-BBD4-8BA71C7E537F}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="14.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.23046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -965,7 +975,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -984,14 +994,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAC09EB0-D87C-4E41-BE46-78AEA78D54B3}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="8.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.765625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.53515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1002,18 +1012,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>4</v>
+      <c r="B2" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="C2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1024,7 +1034,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1035,7 +1045,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1046,7 +1056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1057,7 +1067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Refactor is complete for Home and Planning...As stated on status email only that part need to modify
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{938EDAA3-1C44-4F16-840B-883887063E34}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF98F3DC-ACC4-440A-A245-2F1F06519BB1}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="4" activeTab="7" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="3" activeTab="4" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="1" r:id="rId1"/>
@@ -781,12 +781,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E2F0B9B-0D1C-441E-8138-8347B90B311F}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.53125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
@@ -811,8 +811,18 @@
         <v>29467</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B3" s="5"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B4" s="5"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B6" s="5"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
1. Completed 9 test cases frp RnR functionality 2. Completed 3 test cases for UAT (Added newly feature and Properties file for UAT)
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalOrganization_Field_Values.xlsx
+++ b/src/main/resources/InternalOrganization_Field_Values.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCAE9D93-4A9E-4E4B-9FBD-D057FD9E13FC}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAFAC54-DEB8-45AE-A5B8-8ACA0BCE8046}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="3" activeTab="5" xr2:uid="{2ADB9D40-81FB-44F5-AC46-A89B5F4E8BDF}"/>
   </bookViews>
@@ -118,9 +118,6 @@
     <t>Primary</t>
   </si>
   <si>
-    <t>MailingCountry</t>
-  </si>
-  <si>
     <t>USA</t>
   </si>
   <si>
@@ -130,12 +127,6 @@
     <t>MailingCity</t>
   </si>
   <si>
-    <t>MailingState</t>
-  </si>
-  <si>
-    <t>MailingPostalCode</t>
-  </si>
-  <si>
     <t>Contact</t>
   </si>
   <si>
@@ -179,6 +170,15 @@
   </si>
   <si>
     <t>fieldMailingStreet</t>
+  </si>
+  <si>
+    <t>fieldMailingCountry</t>
+  </si>
+  <si>
+    <t>fieldMailingPostalCode</t>
+  </si>
+  <si>
+    <t>fieldState__c</t>
   </si>
 </sst>
 </file>
@@ -588,7 +588,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -599,7 +599,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -610,7 +610,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
@@ -854,7 +854,7 @@
         <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -865,7 +865,7 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -898,7 +898,7 @@
         <v>26</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -906,7 +906,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s">
         <v>19</v>
@@ -917,7 +917,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
@@ -928,7 +928,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -939,7 +939,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="C10">
         <v>20171</v>
@@ -950,10 +950,10 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
         <v>28</v>
-      </c>
-      <c r="C11" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1027,10 +1027,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -1038,7 +1038,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C3">
         <v>20</v>
@@ -1049,10 +1049,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
@@ -1060,7 +1060,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -1071,7 +1071,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -1082,10 +1082,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>